<commit_message>
Doc(jdt): jdt Thomas P
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_PeltierThomas.xlsx
+++ b/Doc/Journal-de-Travail_PeltierThomas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv03xgo\Documents\GitHub\secured_webshop\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052B474F-DBFC-497A-8627-6D3CCD8650CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1946D72-9C22-4D88-A5DB-C4455B82317B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="3630" yWindow="1110" windowWidth="23070" windowHeight="13395" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="53">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t>J'ai avancé sur le rapport</t>
+  </si>
+  <si>
+    <t>TEST aural</t>
+  </si>
+  <si>
+    <t>J'ai fini mon rapport</t>
   </si>
 </sst>
 </file>
@@ -1201,7 +1207,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>15</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>910</c:v>
@@ -1210,7 +1216,7 @@
                   <c:v>90</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>345</c:v>
+                  <c:v>525</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>225</c:v>
@@ -2056,16 +2062,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>9.4637223974763408E-3</c:v>
+                  <c:v>3.3149171270718231E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.57413249211356465</c:v>
+                  <c:v>0.50276243093922657</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.6782334384858045E-2</c:v>
+                  <c:v>4.9723756906077346E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.21766561514195584</c:v>
+                  <c:v>0.29005524861878451</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4300,7 +4306,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>26 heures 25 minutes</v>
+        <v>30 heures 10 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4315,15 +4321,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>1140</v>
+        <v>1320</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>445</v>
+        <v>490</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1585</v>
+        <v>1810</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4857,27 +4863,45 @@
       <c r="G26" s="39"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="63" t="str">
+      <c r="A27" s="63">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="34"/>
+        <v>21</v>
+      </c>
+      <c r="B27" s="34">
+        <v>46162</v>
+      </c>
       <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="23"/>
+      <c r="D27" s="36">
+        <v>45</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G27" s="40"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="62" t="str">
+      <c r="A28" s="62">
         <f>IF(ISBLANK(B28),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="22"/>
+        <v>21</v>
+      </c>
+      <c r="B28" s="30">
+        <v>46162</v>
+      </c>
+      <c r="C28" s="31">
+        <v>3</v>
+      </c>
+      <c r="D28" s="32">
+        <v>0</v>
+      </c>
+      <c r="E28" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" s="22" t="s">
+        <v>52</v>
+      </c>
       <c r="G28" s="39"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -11066,11 +11090,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11078,11 +11102,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 15 min</v>
+        <v>1 h 00 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>9.4637223974763408E-3</v>
+        <v>3.3149171270718231E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11119,7 +11143,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.57413249211356465</v>
+        <v>0.50276243093922657</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11156,7 +11180,7 @@
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>5.6782334384858045E-2</v>
+        <v>4.9723756906077346E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11173,7 +11197,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>300</v>
+        <v>480</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
@@ -11181,7 +11205,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>345</v>
+        <v>525</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11189,11 +11213,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 45 min</v>
+        <v>8 h 45 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.21766561514195584</v>
+        <v>0.29005524861878451</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11229,7 +11253,7 @@
       </c>
       <c r="G10" s="80">
         <f>SUM(A10:B10)/$C$11</f>
-        <v>0.14195583596214512</v>
+        <v>0.12430939226519337</v>
       </c>
       <c r="L10" s="69" t="s">
         <v>17</v>
@@ -11245,26 +11269,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>1140</v>
+        <v>1320</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>445</v>
+        <v>490</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1585</v>
+        <v>1810</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>26 h 25 min</v>
+        <v>30 h 10 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.29351851851851851</v>
+        <v>0.3351851851851852</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11303,6 +11327,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="5bf905bc6027d3a3176cf398b6d748a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc8923a5f0a5cb2ad217e59a32ed26c" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11491,17 +11526,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11512,6 +11536,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB23EBB1-226D-48F9-BD4F-72DBF2899D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11530,17 +11565,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>